<commit_message>
erreur de rendu réparée et rendu regénéré
</commit_message>
<xml_diff>
--- a/docs/downloads/04/tbl_cm_educ_alaotra_ambatoharanana.xlsx
+++ b/docs/downloads/04/tbl_cm_educ_alaotra_ambatoharanana.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -384,7 +384,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Inconnu</t>
+          <t>Non scolarisé</t>
         </is>
       </c>
     </row>
@@ -436,10 +436,10 @@
         </is>
       </c>
       <c r="C5">
-        <v>51</v>
+        <v>11</v>
       </c>
       <c r="D5">
-        <v>10.1</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="6">
@@ -450,14 +450,14 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Primaire</t>
+          <t>Non scolarisé</t>
         </is>
       </c>
       <c r="C6">
-        <v>307</v>
+        <v>40</v>
       </c>
       <c r="D6">
-        <v>60.6</v>
+        <v>7.9</v>
       </c>
     </row>
     <row r="7">
@@ -468,14 +468,14 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Secondaire 1er cycle</t>
+          <t>Primaire</t>
         </is>
       </c>
       <c r="C7">
-        <v>109</v>
+        <v>307</v>
       </c>
       <c r="D7">
-        <v>21.5</v>
+        <v>60.6</v>
       </c>
     </row>
     <row r="8">
@@ -486,13 +486,31 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
+          <t>Secondaire 1er cycle</t>
+        </is>
+      </c>
+      <c r="C8">
+        <v>109</v>
+      </c>
+      <c r="D8">
+        <v>21.5</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Alaotra - Tous</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
           <t>Secondaire 2ème cycle &amp; sup.</t>
         </is>
       </c>
-      <c r="C8">
+      <c r="C9">
         <v>40</v>
       </c>
-      <c r="D8">
+      <c r="D9">
         <v>7.9</v>
       </c>
     </row>

</xml_diff>